<commit_message>
Checkpoint: Checkpoint saved: Procesador de folios pendientes corregido y funcionando
✅ NUEVO: Procesamiento correcto de archivo de folios pendientes
- Analizadoestructura real del archivo proporcionado (Concepto, Folio, Fecha, Vence, Atraso, Saldo)
- Corregido procesador xlsxProcessor.ts para reconocer formato real
- Procesamiento exitoso: 211 folios pendientes de 839 registros
- Lógica implementada: Si el folio aparece en este archivo = NO PAGADO
- Plantilla Excel actualizada con formato correcto
- Documentación actualizada en interfaz de usuario
- Pruebas realizadas con archivo real del usuario

Funcionalidades previas mantenidas:
✅ Sistema libre de duplicados con validaciones
✅ Plantillas Excel para carga de datos
✅ Control de acceso por dominio
✅ Módulo de administración de usuarios con roles
✅ Gestión completa de clientes y grupos
✅ Sistema de proyección de facturación mensual
✅ Dashboard con métricas y visualizaciones
✅ 81 tests unitarios pasando
</commit_message>
<xml_diff>
--- a/client/public/templates/plantilla_pendientes.xlsx
+++ b/client/public/templates/plantilla_pendientes.xlsx
@@ -1,91 +1,55 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet sheetId="1" name="Pendientes de Pago" state="visible" r:id="rId4"/>
+    <sheet name="Pendientes" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>Folio</t>
-  </si>
-  <si>
-    <t>Cliente</t>
-  </si>
-  <si>
-    <t>Alias</t>
-  </si>
-  <si>
-    <t>Descripción</t>
-  </si>
-  <si>
-    <t>Días Vencido</t>
-  </si>
-  <si>
-    <t>Saldo</t>
-  </si>
-  <si>
-    <t>AB6599</t>
-  </si>
-  <si>
-    <t>EMBUTIDOS SAN LUIS</t>
-  </si>
-  <si>
-    <t>EMBUTIDOS</t>
-  </si>
-  <si>
-    <t>Factura pendiente de pago</t>
-  </si>
-  <si>
-    <t>AA1234</t>
-  </si>
-  <si>
-    <t>PANADERIA LA SUPERIOR</t>
-  </si>
-  <si>
-    <t>PANADERIA</t>
-  </si>
-  <si>
-    <t>Factura vencida</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFED7D31"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -100,25 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -443,80 +396,72 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="80" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15" style="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Concepto</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Folio</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Fecha</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Vence</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Atraso</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Saldo</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Venta</v>
+      </c>
+      <c r="B2" t="str">
+        <v>AB12345</v>
+      </c>
+      <c r="C2" t="str">
+        <v>01/02/2026</v>
+      </c>
+      <c r="D2" t="str">
+        <v>15/02/2026</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Venta</v>
+      </c>
+      <c r="B3" t="str">
+        <v>AA67890</v>
+      </c>
+      <c r="C3" t="str">
+        <v>05/02/2026</v>
+      </c>
+      <c r="D3" t="str">
+        <v>20/02/2026</v>
+      </c>
+      <c r="E3">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2">
-        <v>15</v>
-      </c>
-      <c r="F2" s="1">
-        <v>7920.49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3">
-        <v>30</v>
-      </c>
-      <c r="F3" s="1">
-        <v>10090</v>
+      <c r="F3">
+        <v>8500.5</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>